<commit_message>
Adding the calendar anomaly in mcp
</commit_message>
<xml_diff>
--- a/KG/Batch_KG/sample_data/class_level_data_1.xlsx
+++ b/KG/Batch_KG/sample_data/class_level_data_1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Iris\practice\GenAI\code\Batch_KG\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F06662E-3E53-408D-A0F4-195405F09018}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D1B6364-EAFE-4C6C-9739-F084CFE549D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="736" firstSheet="5" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="736" firstSheet="4" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="JobGroups" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1142" uniqueCount="565">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1136" uniqueCount="566">
   <si>
     <t>id</t>
   </si>
@@ -339,9 +339,6 @@
     <t>Weekend Days</t>
   </si>
   <si>
-    <t>Business Hours</t>
-  </si>
-  <si>
     <t>Global Holidays in US</t>
   </si>
   <si>
@@ -1539,9 +1536,6 @@
     <t>New Year and Christmas</t>
   </si>
   <si>
-    <t>{"holidayNames": ["New Year's Day", "Christmas Day"]}</t>
-  </si>
-  <si>
     <t>RULE_TUE_TO_SAT</t>
   </si>
   <si>
@@ -1741,6 +1735,15 @@
   </si>
   <si>
     <t>Independence Day</t>
+  </si>
+  <si>
+    <t>JG_EOD,JG_TEST</t>
+  </si>
+  <si>
+    <t>JG_EOD,JG_MID</t>
+  </si>
+  <si>
+    <t>{"holidayDates": ["2026-01-01", "2026-12-25"]}</t>
   </si>
 </sst>
 </file>
@@ -2230,13 +2233,13 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>267</v>
+      </c>
+      <c r="B3" t="s">
         <v>268</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>269</v>
-      </c>
-      <c r="C3" t="s">
-        <v>270</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
@@ -2250,13 +2253,13 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>286</v>
+      </c>
+      <c r="B4" t="s">
         <v>287</v>
       </c>
-      <c r="B4" t="s">
-        <v>288</v>
-      </c>
       <c r="C4" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
@@ -2265,18 +2268,18 @@
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B5" t="s">
+        <v>298</v>
+      </c>
+      <c r="C5" t="s">
         <v>299</v>
-      </c>
-      <c r="C5" t="s">
-        <v>300</v>
       </c>
       <c r="D5" t="s">
         <v>8</v>
@@ -2285,18 +2288,18 @@
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>324</v>
+      </c>
+      <c r="B6" t="s">
         <v>325</v>
       </c>
-      <c r="B6" t="s">
-        <v>326</v>
-      </c>
       <c r="C6" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
@@ -2330,28 +2333,28 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>173</v>
-      </c>
       <c r="D1" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>201</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>202</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>2</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>180</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>181</v>
       </c>
       <c r="J1" s="7" t="s">
         <v>4</v>
@@ -2359,31 +2362,31 @@
     </row>
     <row r="2" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C2" t="s">
         <v>68</v>
       </c>
       <c r="D2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E2" t="s">
         <v>22</v>
       </c>
       <c r="F2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="H2" t="s">
+        <v>185</v>
+      </c>
+      <c r="I2" t="s">
         <v>186</v>
-      </c>
-      <c r="I2" t="s">
-        <v>187</v>
       </c>
       <c r="J2" t="b">
         <v>1</v>
@@ -2391,31 +2394,31 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C3" t="s">
         <v>68</v>
       </c>
       <c r="D3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H3" t="s">
+        <v>185</v>
+      </c>
+      <c r="I3" t="s">
         <v>186</v>
-      </c>
-      <c r="I3" t="s">
-        <v>187</v>
       </c>
       <c r="J3" t="b">
         <v>1</v>
@@ -2423,31 +2426,31 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C4" t="s">
         <v>68</v>
       </c>
       <c r="D4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="J4" t="b">
         <v>1</v>
@@ -2455,31 +2458,31 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B5" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C5" t="s">
         <v>68</v>
       </c>
       <c r="D5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F5" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="J5" t="b">
         <v>1</v>
@@ -2487,28 +2490,28 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C6" t="s">
         <v>68</v>
       </c>
       <c r="D6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E6" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="H6" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="J6" t="b">
         <v>1</v>
@@ -2516,28 +2519,28 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B7" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C7" t="s">
         <v>68</v>
       </c>
       <c r="D7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E7" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F7" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="H7" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="J7" t="b">
         <v>1</v>
@@ -2545,31 +2548,31 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B8" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C8" t="s">
         <v>68</v>
       </c>
       <c r="D8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E8" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F8" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="H8" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="I8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="J8" t="b">
         <v>1</v>
@@ -2583,7 +2586,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05669172-4566-411C-BAD9-C6B812325413}">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.6328125" bestFit="1" customWidth="1"/>
@@ -2609,18 +2612,18 @@
         <v>92</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="B2" t="s">
         <v>96</v>
@@ -2640,16 +2643,16 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B3" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>80</v>
       </c>
       <c r="D3" t="s">
-        <v>5</v>
+        <v>563</v>
       </c>
       <c r="E3" t="s">
         <v>95</v>
@@ -2660,33 +2663,33 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>80</v>
       </c>
       <c r="D4" t="s">
-        <v>5</v>
+        <v>564</v>
       </c>
       <c r="E4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="B5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>80</v>
@@ -2695,21 +2698,21 @@
         <v>5</v>
       </c>
       <c r="E5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
       </c>
       <c r="G5" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>80</v>
@@ -2718,50 +2721,47 @@
         <v>5</v>
       </c>
       <c r="E6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
       </c>
       <c r="G6" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>80</v>
       </c>
       <c r="D7" t="s">
-        <v>268</v>
+        <v>286</v>
       </c>
       <c r="E7" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
-      </c>
-      <c r="G7" t="s">
-        <v>481</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>452</v>
+        <v>434</v>
       </c>
       <c r="B8" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>80</v>
       </c>
       <c r="D8" t="s">
-        <v>287</v>
+        <v>267</v>
       </c>
       <c r="E8" t="s">
         <v>95</v>
@@ -2772,65 +2772,45 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>435</v>
+        <v>494</v>
       </c>
       <c r="B9" t="s">
-        <v>101</v>
+        <v>495</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>80</v>
       </c>
       <c r="D9" t="s">
-        <v>268</v>
+        <v>286</v>
       </c>
       <c r="E9" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="F9" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G9" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>435</v>
+        <v>451</v>
       </c>
       <c r="B10" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="D10" t="s">
-        <v>287</v>
+        <v>142</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>335</v>
       </c>
       <c r="E10" t="s">
         <v>95</v>
       </c>
       <c r="F10" t="b">
         <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>495</v>
-      </c>
-      <c r="B11" t="s">
-        <v>496</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="D11" t="s">
-        <v>287</v>
-      </c>
-      <c r="E11" t="s">
-        <v>103</v>
-      </c>
-      <c r="F11" t="b">
-        <v>1</v>
-      </c>
-      <c r="G11" t="s">
-        <v>481</v>
       </c>
     </row>
   </sheetData>
@@ -2858,7 +2838,7 @@
         <v>82</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>1</v>
@@ -2866,338 +2846,338 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B2" s="9">
         <v>46023</v>
       </c>
       <c r="C2" s="9" t="s">
+        <v>359</v>
+      </c>
+      <c r="D2" t="s">
         <v>360</v>
-      </c>
-      <c r="D2" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B3" s="9">
         <v>46023</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D3" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B4" s="9">
         <v>46023</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D4" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B5" s="9">
         <v>46041</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B6" s="9">
         <v>46069</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D6" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B7" s="9">
         <v>46115</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D7" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B8" s="9">
         <v>46160</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D8" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B9" s="9">
         <v>46167</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D9" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B10" s="9">
         <v>46192</v>
       </c>
       <c r="C10" s="9" t="s">
+        <v>345</v>
+      </c>
+      <c r="D10" t="s">
         <v>346</v>
-      </c>
-      <c r="D10" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B11" s="9">
         <v>46204</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D11" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B12" s="9">
         <v>46207</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D12" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B13" s="9">
         <v>46272</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D13" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B14" s="9">
         <v>46272</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D14" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B15" s="9">
         <v>46272</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D15" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B16" s="9">
         <v>46295</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D16" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B17" s="9">
         <v>46307</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D17" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B18" s="9">
         <v>46307</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D18" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B19" s="9">
         <v>46337</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D19" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B20" s="9">
         <v>46337</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D20" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="B21" s="9">
         <v>46352</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D21" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B22" s="9">
         <v>46381</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D22" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="B23" s="9">
         <v>46381</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D23" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="B24" s="9">
         <v>46381</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D24" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="B25" s="9">
         <v>46382</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D25" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
   </sheetData>
@@ -3225,7 +3205,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>4</v>
@@ -3236,376 +3216,376 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D2" t="b">
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D3" t="b">
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D4" t="b">
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D5" t="b">
         <v>1</v>
       </c>
       <c r="E5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B6" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D6" t="b">
         <v>1</v>
       </c>
       <c r="E6" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
+        <v>231</v>
+      </c>
+      <c r="B7" t="s">
+        <v>158</v>
+      </c>
+      <c r="C7" t="s">
         <v>232</v>
       </c>
-      <c r="B7" t="s">
-        <v>159</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="D7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" t="s">
         <v>233</v>
-      </c>
-      <c r="D7" t="b">
-        <v>1</v>
-      </c>
-      <c r="E7" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B8" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D8" t="b">
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B9" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D9" t="b">
         <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B10" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D10" t="b">
         <v>1</v>
       </c>
       <c r="E10" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B11" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D11" t="b">
         <v>1</v>
       </c>
       <c r="E11" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B12" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C12" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D12" t="b">
         <v>1</v>
       </c>
       <c r="E12" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B13" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D13" t="b">
         <v>1</v>
       </c>
       <c r="E13" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B14" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C14" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D14" t="b">
         <v>1</v>
       </c>
       <c r="E14" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
+        <v>273</v>
+      </c>
+      <c r="B15" t="s">
         <v>274</v>
       </c>
-      <c r="B15" t="s">
-        <v>275</v>
-      </c>
       <c r="C15" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D15" t="b">
         <v>1</v>
       </c>
       <c r="E15" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B16" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C16" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D16" t="b">
         <v>1</v>
       </c>
       <c r="E16" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B17" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C17" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D17" t="b">
         <v>1</v>
       </c>
       <c r="E17" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B18" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C18" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D18" t="b">
         <v>1</v>
       </c>
       <c r="E18" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B19" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C19" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D19" t="b">
         <v>1</v>
       </c>
       <c r="E19" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B20" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C20" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D20" t="b">
         <v>1</v>
       </c>
       <c r="E20" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B21" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C21" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D21" t="b">
         <v>1</v>
       </c>
       <c r="E21" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B22" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C22" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D22" t="b">
         <v>1</v>
       </c>
       <c r="E22" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B23" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C23" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D23" t="b">
         <v>1</v>
       </c>
       <c r="E23" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
   </sheetData>
@@ -3633,170 +3613,170 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>178</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>179</v>
       </c>
       <c r="I1" s="6" t="s">
         <v>2</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>180</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B2" t="s">
         <v>68</v>
       </c>
       <c r="C2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E2" t="s">
+        <v>182</v>
+      </c>
+      <c r="F2" t="s">
+        <v>164</v>
+      </c>
+      <c r="G2" t="s">
         <v>183</v>
       </c>
-      <c r="F2" t="s">
-        <v>165</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>184</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="J2" t="s">
         <v>185</v>
       </c>
-      <c r="I2" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>186</v>
-      </c>
-      <c r="K2" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B3" t="s">
         <v>68</v>
       </c>
       <c r="C3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G3" t="s">
+        <v>188</v>
+      </c>
+      <c r="H3" t="s">
         <v>189</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="J3" t="s">
+        <v>185</v>
+      </c>
+      <c r="K3" t="s">
         <v>190</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="J3" t="s">
-        <v>186</v>
-      </c>
-      <c r="K3" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B4" t="s">
         <v>68</v>
       </c>
       <c r="D4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E4" t="s">
+        <v>182</v>
+      </c>
+      <c r="F4" t="s">
+        <v>162</v>
+      </c>
+      <c r="G4" t="s">
         <v>183</v>
       </c>
-      <c r="F4" t="s">
-        <v>163</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>184</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="J4" t="s">
         <v>185</v>
       </c>
-      <c r="I4" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="J4" t="s">
-        <v>186</v>
-      </c>
       <c r="K4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B5" t="s">
         <v>68</v>
       </c>
       <c r="C5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D5" t="s">
+        <v>183</v>
+      </c>
+      <c r="E5" t="s">
+        <v>182</v>
+      </c>
+      <c r="F5" t="s">
+        <v>160</v>
+      </c>
+      <c r="G5" t="s">
+        <v>183</v>
+      </c>
+      <c r="H5" t="s">
         <v>184</v>
       </c>
-      <c r="E5" t="s">
-        <v>183</v>
-      </c>
-      <c r="F5" t="s">
-        <v>161</v>
-      </c>
-      <c r="G5" t="s">
-        <v>184</v>
-      </c>
-      <c r="H5" t="s">
-        <v>185</v>
-      </c>
       <c r="J5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="J6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
   </sheetData>
@@ -3832,7 +3812,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
@@ -3973,13 +3953,13 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
+        <v>326</v>
+      </c>
+      <c r="B10" t="s">
+        <v>326</v>
+      </c>
+      <c r="C10" t="s">
         <v>327</v>
-      </c>
-      <c r="B10" t="s">
-        <v>327</v>
-      </c>
-      <c r="C10" t="s">
-        <v>328</v>
       </c>
       <c r="D10" t="b">
         <v>1</v>
@@ -3990,13 +3970,13 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
+        <v>328</v>
+      </c>
+      <c r="B11" t="s">
+        <v>328</v>
+      </c>
+      <c r="C11" t="s">
         <v>329</v>
-      </c>
-      <c r="B11" t="s">
-        <v>329</v>
-      </c>
-      <c r="C11" t="s">
-        <v>330</v>
       </c>
       <c r="D11" t="b">
         <v>1</v>
@@ -4007,13 +3987,13 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
+        <v>330</v>
+      </c>
+      <c r="B12" t="s">
+        <v>330</v>
+      </c>
+      <c r="C12" t="s">
         <v>331</v>
-      </c>
-      <c r="B12" t="s">
-        <v>331</v>
-      </c>
-      <c r="C12" t="s">
-        <v>332</v>
       </c>
       <c r="D12" t="b">
         <v>1</v>
@@ -4024,13 +4004,13 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
+        <v>332</v>
+      </c>
+      <c r="B13" t="s">
+        <v>332</v>
+      </c>
+      <c r="C13" t="s">
         <v>333</v>
-      </c>
-      <c r="B13" t="s">
-        <v>333</v>
-      </c>
-      <c r="C13" t="s">
-        <v>334</v>
       </c>
       <c r="D13" t="b">
         <v>1</v>
@@ -4057,7 +4037,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>9</v>
@@ -4132,7 +4112,7 @@
         <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
@@ -4140,7 +4120,7 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
@@ -4148,7 +4128,7 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
@@ -4156,7 +4136,7 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
@@ -4164,7 +4144,7 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
@@ -4172,7 +4152,7 @@
         <v>15</v>
       </c>
       <c r="B15" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
@@ -4180,7 +4160,7 @@
         <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -4188,7 +4168,7 @@
         <v>18</v>
       </c>
       <c r="B17" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -4196,7 +4176,7 @@
         <v>12</v>
       </c>
       <c r="B18" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
@@ -4204,7 +4184,7 @@
         <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -4212,7 +4192,7 @@
         <v>14</v>
       </c>
       <c r="B20" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
@@ -4220,7 +4200,7 @@
         <v>16</v>
       </c>
       <c r="B21" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
@@ -4228,47 +4208,47 @@
         <v>11</v>
       </c>
       <c r="B22" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B23" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B24" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B25" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B26" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B27" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
   </sheetData>
@@ -4303,10 +4283,10 @@
         <v>19</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>20</v>
@@ -4315,7 +4295,7 @@
         <v>4</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="I1" s="7" t="s">
         <v>2</v>
@@ -4323,10 +4303,10 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C2" t="s">
         <v>22</v>
@@ -4341,15 +4321,15 @@
         <v>1</v>
       </c>
       <c r="H2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C3" t="s">
         <v>22</v>
@@ -4364,15 +4344,15 @@
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C4" t="s">
         <v>22</v>
@@ -4387,15 +4367,15 @@
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C5" t="s">
         <v>22</v>
@@ -4410,15 +4390,15 @@
         <v>1</v>
       </c>
       <c r="H5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C6" t="s">
         <v>22</v>
@@ -4433,15 +4413,15 @@
         <v>1</v>
       </c>
       <c r="H6" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C7" t="s">
         <v>22</v>
@@ -4456,12 +4436,12 @@
         <v>1</v>
       </c>
       <c r="H7" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>29</v>
@@ -4479,12 +4459,12 @@
         <v>1</v>
       </c>
       <c r="H8" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>31</v>
@@ -4502,12 +4482,12 @@
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>33</v>
@@ -4525,12 +4505,12 @@
         <v>1</v>
       </c>
       <c r="H10" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>35</v>
@@ -4548,12 +4528,12 @@
         <v>1</v>
       </c>
       <c r="H11" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>37</v>
@@ -4571,12 +4551,12 @@
         <v>1</v>
       </c>
       <c r="H12" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>39</v>
@@ -4594,12 +4574,12 @@
         <v>1</v>
       </c>
       <c r="H13" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>41</v>
@@ -4617,12 +4597,12 @@
         <v>1</v>
       </c>
       <c r="H14" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>43</v>
@@ -4640,12 +4620,12 @@
         <v>1</v>
       </c>
       <c r="H15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>45</v>
@@ -4663,187 +4643,187 @@
         <v>1</v>
       </c>
       <c r="H16" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B17" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C17" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E17" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G17" t="b">
         <v>1</v>
       </c>
       <c r="H17" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B18" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C18" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E18" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G18" t="b">
         <v>1</v>
       </c>
       <c r="H18" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B19" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C19" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E19" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G19" t="b">
         <v>1</v>
       </c>
       <c r="H19" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B20" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E20" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G20" t="b">
         <v>1</v>
       </c>
       <c r="H20" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B21" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C21" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E21" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G21" t="b">
         <v>1</v>
       </c>
       <c r="H21" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B22" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C22" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E22" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G22" t="b">
         <v>1</v>
       </c>
       <c r="H22" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B23" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C23" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E23" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G23" t="b">
         <v>1</v>
       </c>
       <c r="H23" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
+        <v>228</v>
+      </c>
+      <c r="B24" t="s">
+        <v>170</v>
+      </c>
+      <c r="C24" t="s">
         <v>229</v>
       </c>
-      <c r="B24" t="s">
-        <v>171</v>
-      </c>
-      <c r="C24" t="s">
-        <v>230</v>
-      </c>
       <c r="E24" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G24" t="b">
         <v>1</v>
       </c>
       <c r="H24" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
+        <v>339</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>340</v>
       </c>
-      <c r="B25" s="3" t="s">
-        <v>341</v>
-      </c>
       <c r="C25" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E25" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="G25" t="b">
         <v>1</v>
       </c>
       <c r="H25" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>
@@ -4880,7 +4860,7 @@
         <v>94</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
@@ -4908,7 +4888,7 @@
         <v>86</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
@@ -4925,7 +4905,7 @@
         <v>86</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
@@ -4942,7 +4922,7 @@
         <v>87</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
@@ -4959,7 +4939,7 @@
         <v>88</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
@@ -4976,7 +4956,7 @@
         <v>89</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
@@ -4993,7 +4973,7 @@
         <v>91</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="29" x14ac:dyDescent="0.35">
@@ -5010,10 +4990,10 @@
         <v>95</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
@@ -5030,344 +5010,344 @@
         <v>83</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>17</v>
       </c>
       <c r="C11" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C13" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>14</v>
       </c>
       <c r="C14" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>16</v>
       </c>
       <c r="C15" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C16" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>15</v>
       </c>
       <c r="C17" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C18" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>95</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>18</v>
       </c>
       <c r="C19" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C20" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C21" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>14</v>
       </c>
       <c r="C22" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>16</v>
       </c>
       <c r="C23" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C24" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C25" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>95</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C26" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>95</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="B27" t="s">
+        <v>326</v>
+      </c>
+      <c r="C27" t="s">
+        <v>324</v>
+      </c>
+      <c r="E27" s="3" t="s">
         <v>336</v>
       </c>
-      <c r="B27" t="s">
-        <v>327</v>
-      </c>
-      <c r="C27" t="s">
-        <v>325</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>337</v>
-      </c>
       <c r="F27" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="B28" t="s">
+        <v>328</v>
+      </c>
+      <c r="C28" t="s">
+        <v>324</v>
+      </c>
+      <c r="E28" s="3" t="s">
         <v>337</v>
       </c>
-      <c r="B28" t="s">
-        <v>329</v>
-      </c>
-      <c r="C28" t="s">
-        <v>325</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>338</v>
-      </c>
       <c r="F28" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B29" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C29" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B30" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C30" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -5404,21 +5384,21 @@
         <v>4</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>90</v>
@@ -5427,21 +5407,21 @@
         <v>1</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>80</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E3" t="s">
         <v>5</v>
@@ -5450,21 +5430,21 @@
         <v>1</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>86</v>
@@ -5473,21 +5453,21 @@
         <v>1</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>80</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E5" t="s">
         <v>5</v>
@@ -5496,53 +5476,53 @@
         <v>1</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>80</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E6" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="F6" s="3" t="b">
         <v>1</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>80</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E7" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F7" s="3" t="b">
         <v>1</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -5580,13 +5560,13 @@
         <v>51</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>52</v>
@@ -5618,7 +5598,7 @@
         <v>360000</v>
       </c>
       <c r="H2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I2" t="s">
         <v>70</v>
@@ -5644,7 +5624,7 @@
         <v>300000</v>
       </c>
       <c r="H3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I3" t="s">
         <v>70</v>
@@ -5670,7 +5650,7 @@
         <v>420000</v>
       </c>
       <c r="H4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I4" t="s">
         <v>70</v>
@@ -5693,16 +5673,16 @@
         <v>74</v>
       </c>
       <c r="D5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F5">
         <v>600000</v>
       </c>
       <c r="H5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I5" t="s">
         <v>70</v>
@@ -5728,7 +5708,7 @@
         <v>300000</v>
       </c>
       <c r="H6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I6" t="s">
         <v>70</v>
@@ -5754,7 +5734,7 @@
         <v>540000</v>
       </c>
       <c r="H7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I7" t="s">
         <v>70</v>
@@ -5780,7 +5760,7 @@
         <v>240000</v>
       </c>
       <c r="H8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I8" t="s">
         <v>70</v>
@@ -5806,7 +5786,7 @@
         <v>360000</v>
       </c>
       <c r="H9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I9" t="s">
         <v>70</v>
@@ -5832,7 +5812,7 @@
         <v>3600000</v>
       </c>
       <c r="H10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I10" t="s">
         <v>70</v>
@@ -5852,7 +5832,7 @@
         <v>65</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>48</v>
@@ -5861,16 +5841,16 @@
         <v>47</v>
       </c>
       <c r="H11" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I11" t="s">
         <v>8</v>
       </c>
       <c r="J11" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L11" t="b">
         <v>1</v>
@@ -5881,7 +5861,7 @@
         <v>66</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>48</v>
@@ -5890,16 +5870,16 @@
         <v>47</v>
       </c>
       <c r="H12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I12" t="s">
         <v>8</v>
       </c>
       <c r="J12" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K12" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="L12" t="b">
         <v>1</v>
@@ -5910,25 +5890,25 @@
         <v>67</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G13" t="s">
         <v>47</v>
       </c>
       <c r="H13" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I13" t="s">
         <v>8</v>
       </c>
       <c r="J13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K13" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="L13" t="b">
         <v>1</v>
@@ -5936,10 +5916,10 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>48</v>
@@ -5948,16 +5928,16 @@
         <v>47</v>
       </c>
       <c r="H14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I14" t="s">
         <v>8</v>
       </c>
       <c r="J14" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K14" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L14" t="b">
         <v>1</v>
@@ -5965,10 +5945,10 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B15" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C15" s="8">
         <v>0.29236111111111113</v>
@@ -5977,7 +5957,7 @@
         <v>47</v>
       </c>
       <c r="H15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I15" t="s">
         <v>8</v>
@@ -5986,7 +5966,7 @@
         <v>80</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="L15" t="b">
         <v>1</v>
@@ -5994,16 +5974,16 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B16" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F16">
         <v>3200000</v>
       </c>
       <c r="H16" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I16" t="s">
         <v>70</v>
@@ -6012,7 +5992,7 @@
         <v>80</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="L16" t="b">
         <v>1</v>
@@ -6020,16 +6000,16 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
+        <v>295</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>296</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>297</v>
       </c>
       <c r="F17">
         <v>60000</v>
       </c>
       <c r="H17" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I17" t="s">
         <v>70</v>
@@ -6038,7 +6018,7 @@
         <v>80</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="L17" t="b">
         <v>1</v>
@@ -6046,16 +6026,16 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="F18">
         <v>60000</v>
       </c>
       <c r="H18" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I18" t="s">
         <v>70</v>
@@ -6064,7 +6044,7 @@
         <v>80</v>
       </c>
       <c r="K18" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="L18" t="b">
         <v>1</v>
@@ -6090,54 +6070,54 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
+        <v>384</v>
+      </c>
+      <c r="B1" s="13" t="s">
         <v>385</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="C1" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>428</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>429</v>
+      </c>
+      <c r="F1" s="13" t="s">
         <v>386</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="13" t="s">
-        <v>429</v>
-      </c>
-      <c r="E1" s="13" t="s">
-        <v>430</v>
-      </c>
-      <c r="F1" s="13" t="s">
-        <v>387</v>
       </c>
       <c r="G1" s="13" t="s">
         <v>2</v>
       </c>
       <c r="H1" s="13" t="s">
+        <v>387</v>
+      </c>
+      <c r="I1" s="13" t="s">
         <v>388</v>
-      </c>
-      <c r="I1" s="13" t="s">
-        <v>389</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="52" x14ac:dyDescent="0.3">
       <c r="A2" s="14" t="s">
+        <v>389</v>
+      </c>
+      <c r="B2" s="14" t="s">
         <v>390</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="C2" s="14" t="s">
         <v>391</v>
-      </c>
-      <c r="C2" s="14" t="s">
-        <v>392</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>82</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="H2" s="14" t="b">
         <v>1</v>
@@ -6148,25 +6128,25 @@
     </row>
     <row r="3" spans="1:9" ht="52" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="B3" s="14" t="s">
         <v>394</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="C3" s="14" t="s">
         <v>395</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>396</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>82</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="F3" s="14" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="H3" s="14" t="b">
         <v>1</v>
@@ -6177,25 +6157,25 @@
     </row>
     <row r="4" spans="1:9" ht="39" x14ac:dyDescent="0.3">
       <c r="A4" s="14" t="s">
+        <v>396</v>
+      </c>
+      <c r="B4" s="14" t="s">
         <v>397</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="C4" s="14" t="s">
         <v>398</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>399</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>82</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="H4" s="14" t="b">
         <v>1</v>
@@ -6206,25 +6186,25 @@
     </row>
     <row r="5" spans="1:9" ht="65" x14ac:dyDescent="0.3">
       <c r="A5" s="14" t="s">
+        <v>400</v>
+      </c>
+      <c r="B5" s="14" t="s">
         <v>401</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="C5" s="14" t="s">
         <v>402</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="D5" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>504</v>
+      </c>
+      <c r="F5" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="D5" s="14" t="s">
-        <v>420</v>
-      </c>
-      <c r="E5" s="14" t="s">
-        <v>506</v>
-      </c>
-      <c r="F5" s="14" t="s">
-        <v>404</v>
-      </c>
       <c r="G5" s="14" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="H5" s="14" t="b">
         <v>1</v>
@@ -6235,25 +6215,25 @@
     </row>
     <row r="6" spans="1:9" ht="52" x14ac:dyDescent="0.3">
       <c r="A6" s="14" t="s">
+        <v>404</v>
+      </c>
+      <c r="B6" s="14" t="s">
         <v>405</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="C6" s="14" t="s">
         <v>406</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="D6" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="E6" s="14" t="s">
+        <v>505</v>
+      </c>
+      <c r="F6" s="14" t="s">
         <v>407</v>
       </c>
-      <c r="D6" s="14" t="s">
-        <v>420</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>507</v>
-      </c>
-      <c r="F6" s="14" t="s">
-        <v>408</v>
-      </c>
       <c r="G6" s="14" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="H6" s="14" t="b">
         <v>1</v>
@@ -6264,25 +6244,25 @@
     </row>
     <row r="7" spans="1:9" ht="52" x14ac:dyDescent="0.3">
       <c r="A7" s="14" t="s">
+        <v>408</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>409</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="C7" s="14" t="s">
         <v>410</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="D7" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>506</v>
+      </c>
+      <c r="F7" s="14" t="s">
         <v>411</v>
       </c>
-      <c r="D7" s="14" t="s">
-        <v>420</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>508</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>412</v>
-      </c>
       <c r="G7" s="14" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="H7" s="14" t="b">
         <v>1</v>
@@ -6293,25 +6273,25 @@
     </row>
     <row r="8" spans="1:9" ht="52" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
+        <v>412</v>
+      </c>
+      <c r="B8" s="14" t="s">
         <v>413</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="C8" s="14" t="s">
         <v>414</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="D8" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>507</v>
+      </c>
+      <c r="F8" s="14" t="s">
         <v>415</v>
       </c>
-      <c r="D8" s="14" t="s">
-        <v>420</v>
-      </c>
-      <c r="E8" s="14" t="s">
-        <v>509</v>
-      </c>
-      <c r="F8" s="14" t="s">
-        <v>416</v>
-      </c>
       <c r="G8" s="14" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="H8" s="14" t="b">
         <v>1</v>
@@ -6322,22 +6302,22 @@
     </row>
     <row r="9" spans="1:9" ht="26" x14ac:dyDescent="0.3">
       <c r="A9" s="14" t="s">
+        <v>416</v>
+      </c>
+      <c r="B9" s="14" t="s">
         <v>417</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="C9" s="14" t="s">
         <v>418</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="D9" s="14" t="s">
         <v>419</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="F9" s="14" t="s">
         <v>420</v>
       </c>
-      <c r="F9" s="14" t="s">
-        <v>421</v>
-      </c>
       <c r="G9" s="14" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="H9" s="14" t="b">
         <v>1</v>
@@ -6348,22 +6328,22 @@
     </row>
     <row r="10" spans="1:9" ht="26" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
+        <v>421</v>
+      </c>
+      <c r="B10" s="14" t="s">
         <v>422</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="C10" s="14" t="s">
         <v>423</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="D10" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="F10" s="14" t="s">
         <v>424</v>
       </c>
-      <c r="D10" s="14" t="s">
-        <v>420</v>
-      </c>
-      <c r="F10" s="14" t="s">
-        <v>425</v>
-      </c>
       <c r="G10" s="14" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="H10" s="14" t="b">
         <v>1</v>
@@ -6374,22 +6354,22 @@
     </row>
     <row r="11" spans="1:9" ht="52" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B11" s="14" t="s">
         <v>81</v>
       </c>
       <c r="C11" s="14" t="s">
+        <v>426</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="F11" s="14" t="s">
         <v>427</v>
       </c>
-      <c r="D11" s="14" t="s">
-        <v>420</v>
-      </c>
-      <c r="F11" s="14" t="s">
-        <v>428</v>
-      </c>
       <c r="G11" s="14" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="H11" s="14" t="b">
         <v>1</v>
@@ -6400,25 +6380,25 @@
     </row>
     <row r="12" spans="1:9" ht="65" x14ac:dyDescent="0.3">
       <c r="A12" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="B12" s="14" t="s">
         <v>458</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="C12" s="14" t="s">
         <v>459</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>460</v>
       </c>
       <c r="D12" s="14" t="s">
         <v>82</v>
       </c>
       <c r="E12" s="14" t="s">
+        <v>460</v>
+      </c>
+      <c r="F12" s="14" t="s">
         <v>461</v>
       </c>
-      <c r="F12" s="14" t="s">
-        <v>462</v>
-      </c>
       <c r="G12" s="14" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="H12" s="14" t="b">
         <v>1</v>
@@ -6429,25 +6409,25 @@
     </row>
     <row r="13" spans="1:9" ht="64" x14ac:dyDescent="0.3">
       <c r="A13" s="14" t="s">
+        <v>484</v>
+      </c>
+      <c r="B13" s="14" t="s">
         <v>485</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="C13" s="14" t="s">
+        <v>490</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>492</v>
+      </c>
+      <c r="F13" s="14" t="s">
         <v>486</v>
       </c>
-      <c r="C13" s="14" t="s">
-        <v>491</v>
-      </c>
-      <c r="D13" s="14" t="s">
-        <v>420</v>
-      </c>
-      <c r="E13" s="14" t="s">
-        <v>493</v>
-      </c>
-      <c r="F13" s="14" t="s">
-        <v>487</v>
-      </c>
       <c r="G13" s="15" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="H13" s="14" t="b">
         <v>1</v>
@@ -6458,25 +6438,25 @@
     </row>
     <row r="14" spans="1:9" ht="48" x14ac:dyDescent="0.3">
       <c r="A14" s="14" t="s">
+        <v>487</v>
+      </c>
+      <c r="B14" s="14" t="s">
         <v>488</v>
       </c>
-      <c r="B14" s="14" t="s">
-        <v>489</v>
-      </c>
       <c r="C14" s="14" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="D14" s="14" t="s">
         <v>82</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="G14" s="15" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="H14" s="14" t="b">
         <v>1</v>
@@ -6506,22 +6486,22 @@
   <sheetData>
     <row r="1" spans="1:7" s="12" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
+        <v>430</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>385</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>383</v>
+      </c>
+      <c r="E1" s="11" t="s">
         <v>431</v>
       </c>
-      <c r="B1" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="11" t="s">
-        <v>386</v>
-      </c>
-      <c r="D1" s="11" t="s">
-        <v>384</v>
-      </c>
-      <c r="E1" s="11" t="s">
-        <v>432</v>
-      </c>
       <c r="F1" s="11" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="G1" s="11" t="s">
         <v>2</v>
@@ -6529,451 +6509,451 @@
     </row>
     <row r="2" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B2" t="s">
         <v>433</v>
       </c>
-      <c r="B2" t="s">
-        <v>434</v>
-      </c>
       <c r="C2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>434</v>
+      </c>
+      <c r="B3" t="s">
         <v>435</v>
       </c>
-      <c r="B3" t="s">
-        <v>436</v>
-      </c>
       <c r="C3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>436</v>
+      </c>
+      <c r="B4" t="s">
         <v>437</v>
       </c>
-      <c r="B4" t="s">
-        <v>438</v>
-      </c>
       <c r="C4" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>438</v>
+      </c>
+      <c r="B5" t="s">
         <v>439</v>
       </c>
-      <c r="B5" t="s">
-        <v>440</v>
-      </c>
       <c r="C5" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>447</v>
+      </c>
+      <c r="B6" t="s">
         <v>448</v>
       </c>
-      <c r="B6" t="s">
-        <v>449</v>
-      </c>
       <c r="C6" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="B7" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="C7" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
+        <v>449</v>
+      </c>
+      <c r="B8" t="s">
         <v>450</v>
       </c>
-      <c r="B8" t="s">
-        <v>451</v>
-      </c>
       <c r="C8" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="F8" t="b">
         <v>1</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
+        <v>440</v>
+      </c>
+      <c r="B9" t="s">
         <v>441</v>
-      </c>
-      <c r="B9" t="s">
-        <v>442</v>
       </c>
       <c r="C9" t="s">
         <v>81</v>
       </c>
       <c r="D9" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F9" t="b">
         <v>1</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
+        <v>443</v>
+      </c>
+      <c r="B10" t="s">
         <v>444</v>
-      </c>
-      <c r="B10" t="s">
-        <v>445</v>
       </c>
       <c r="C10" t="s">
         <v>81</v>
       </c>
       <c r="D10" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F10" t="b">
         <v>1</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
+        <v>451</v>
+      </c>
+      <c r="B11" t="s">
         <v>452</v>
-      </c>
-      <c r="B11" t="s">
-        <v>453</v>
       </c>
       <c r="C11" t="s">
         <v>81</v>
       </c>
       <c r="D11" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F11" t="b">
         <v>1</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
+        <v>453</v>
+      </c>
+      <c r="B12" t="s">
         <v>454</v>
       </c>
-      <c r="B12" t="s">
-        <v>455</v>
-      </c>
       <c r="C12" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="F12" t="b">
         <v>1</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="B13" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="C13" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="F13" t="b">
         <v>1</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
+        <v>455</v>
+      </c>
+      <c r="B14" t="s">
         <v>456</v>
       </c>
-      <c r="B14" t="s">
-        <v>457</v>
-      </c>
       <c r="C14" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="F14" t="b">
         <v>1</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
+        <v>445</v>
+      </c>
+      <c r="B15" t="s">
         <v>446</v>
       </c>
-      <c r="B15" t="s">
-        <v>447</v>
-      </c>
       <c r="C15" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="F15" t="b">
         <v>1</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
+        <v>519</v>
+      </c>
+      <c r="B16" t="s">
         <v>521</v>
       </c>
-      <c r="B16" t="s">
-        <v>523</v>
-      </c>
       <c r="C16" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="F16" t="b">
         <v>1</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
+        <v>462</v>
+      </c>
+      <c r="B17" t="s">
         <v>463</v>
       </c>
-      <c r="B17" t="s">
-        <v>464</v>
-      </c>
       <c r="C17" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="F17" t="b">
         <v>1</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
+        <v>464</v>
+      </c>
+      <c r="B18" t="s">
         <v>465</v>
       </c>
-      <c r="B18" t="s">
-        <v>466</v>
-      </c>
       <c r="C18" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="F18" t="b">
         <v>1</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
+        <v>466</v>
+      </c>
+      <c r="B19" t="s">
         <v>467</v>
       </c>
-      <c r="B19" t="s">
-        <v>468</v>
-      </c>
       <c r="C19" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="F19" t="b">
         <v>1</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
+        <v>468</v>
+      </c>
+      <c r="B20" t="s">
         <v>469</v>
       </c>
-      <c r="B20" t="s">
-        <v>470</v>
-      </c>
       <c r="C20" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="F20" t="b">
         <v>1</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
+        <v>470</v>
+      </c>
+      <c r="B21" t="s">
         <v>471</v>
       </c>
-      <c r="B21" t="s">
-        <v>472</v>
-      </c>
       <c r="C21" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="F21" t="b">
         <v>1</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
+        <v>472</v>
+      </c>
+      <c r="B22" t="s">
         <v>473</v>
       </c>
-      <c r="B22" t="s">
-        <v>474</v>
-      </c>
       <c r="C22" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="F22" t="b">
         <v>1</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
+        <v>494</v>
+      </c>
+      <c r="B23" t="s">
         <v>495</v>
       </c>
-      <c r="B23" t="s">
-        <v>496</v>
-      </c>
       <c r="C23" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>497</v>
+        <v>565</v>
       </c>
       <c r="F23" t="b">
         <v>1</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
     </row>
   </sheetData>

</xml_diff>